<commit_message>
new notification of the customs and dgft
</commit_message>
<xml_diff>
--- a/backend/PDF_DOC/CBIC/Instruction and Guidelines/Instructions and Guidelines.xlsx
+++ b/backend/PDF_DOC/CBIC/Instruction and Guidelines/Instructions and Guidelines.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B510883-ACD7-45E4-84EB-679EC1C8B92B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7E3880E-54F1-4A0D-B3A4-83B32571B715}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026" sheetId="1" r:id="rId1"/>
@@ -509,7 +509,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -528,6 +528,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -541,7 +547,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -588,6 +594,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -868,7 +875,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.28515625" customWidth="1"/>
@@ -876,19 +883,19 @@
     <col min="3" max="3" width="109.85546875" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>127</v>
       </c>
       <c r="C1" s="7"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C2" s="7"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C3" s="7"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -899,7 +906,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
         <v>148</v>
       </c>
@@ -909,13 +916,15 @@
       <c r="C7" s="19" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="D7" s="20"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="17"/>
       <c r="B8" s="17"/>
       <c r="C8" s="19"/>
-    </row>
-    <row r="9" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="D8" s="20"/>
+    </row>
+    <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
         <v>150</v>
       </c>
@@ -925,8 +934,9 @@
       <c r="C9" s="19" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="D9" s="20"/>
+    </row>
+    <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>146</v>
       </c>
@@ -937,7 +947,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>144</v>
       </c>
@@ -948,7 +958,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
         <v>140</v>
       </c>
@@ -959,7 +969,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="10"/>
       <c r="B16" s="13"/>
       <c r="C16" s="11"/>

</xml_diff>

<commit_message>
new notification for the DGFT and CUSTOMS
</commit_message>
<xml_diff>
--- a/backend/PDF_DOC/CBIC/Instruction and Guidelines/Instructions and Guidelines.xlsx
+++ b/backend/PDF_DOC/CBIC/Instruction and Guidelines/Instructions and Guidelines.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58D7BA6A-ED22-47E9-8C1C-13B7A93C6EDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C9EB321-369C-4170-B995-193CA4D2FB2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2026" sheetId="1" r:id="rId1"/>
@@ -522,30 +522,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="2" tint="-0.499984740745262"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -566,7 +548,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -601,27 +583,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="15" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="15" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="15" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -934,81 +921,88 @@
       </c>
     </row>
     <row r="7" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="14" t="s">
         <v>152</v>
       </c>
-      <c r="B7" s="24">
+      <c r="B7" s="17">
         <v>46241</v>
       </c>
-      <c r="C7" s="23" t="s">
+      <c r="C7" s="16" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="21"/>
-      <c r="B8" s="21"/>
-      <c r="C8" s="22"/>
-    </row>
-    <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="17" t="s">
+      <c r="A8" s="14"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="15"/>
+    </row>
+    <row r="9" spans="1:4" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="B9" s="18">
+      <c r="B9" s="19">
         <v>46206</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="20" t="s">
         <v>149</v>
       </c>
-      <c r="D9" s="20"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="17"/>
-      <c r="B10" s="17"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="20"/>
-    </row>
-    <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="17" t="s">
+      <c r="D9" s="21"/>
+    </row>
+    <row r="10" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C10" s="20"/>
+      <c r="D10" s="21"/>
+    </row>
+    <row r="11" spans="1:4" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="18" t="s">
         <v>150</v>
       </c>
-      <c r="B11" s="18">
+      <c r="B11" s="19">
         <v>46206</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="20" t="s">
         <v>151</v>
       </c>
-      <c r="D11" s="20"/>
-    </row>
-    <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="14" t="s">
+      <c r="D11" s="21"/>
+    </row>
+    <row r="12" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C12" s="20"/>
+    </row>
+    <row r="13" spans="1:4" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="22" t="s">
         <v>146</v>
       </c>
-      <c r="B13" s="15">
+      <c r="B13" s="19">
         <v>46196</v>
       </c>
-      <c r="C13" s="16" t="s">
+      <c r="C13" s="20" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="14" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C14" s="20"/>
+    </row>
+    <row r="15" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="18" t="s">
         <v>144</v>
       </c>
-      <c r="B15" s="3">
+      <c r="B15" s="19">
         <v>46191</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="20" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
+    <row r="16" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C16" s="20"/>
+    </row>
+    <row r="17" spans="1:3" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="23" t="s">
         <v>140</v>
       </c>
-      <c r="B17" s="12">
+      <c r="B17" s="24">
         <v>46185</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="C17" s="25" t="s">
         <v>141</v>
       </c>
     </row>
@@ -1028,7 +1022,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>138</v>
       </c>

</xml_diff>